<commit_message>
all purchase related scripts are added.
</commit_message>
<xml_diff>
--- a/Excel-files/Customer_List.xlsx
+++ b/Excel-files/Customer_List.xlsx
@@ -2,15 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BFA904B-5FD8-4BF1-9FB4-6E8F276342F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01503\Documents\load testing Script-BSS\Excel-files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5101F23B-1456-4F5F-ACDD-246F6069AA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19400" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Management" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="0" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -20,29 +25,35 @@
     <t>SID</t>
   </si>
   <si>
-    <t>SID2609000935</t>
+    <t>SID2609000950</t>
   </si>
   <si>
-    <t>SID2609000934</t>
+    <t>SID2609000949</t>
   </si>
   <si>
-    <t>SID2609000933</t>
+    <t>SID2609000948</t>
   </si>
   <si>
-    <t>SID2609000932</t>
+    <t>SID2609000947</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -53,7 +64,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -65,17 +83,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -88,14 +109,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MyTable" displayName="MyTable" ref="A1:A5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MyTable" displayName="MyTable" ref="A1:A5" totalsRowShown="0">
   <autoFilter ref="A1:A5" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SID" totalsRowLabel="Total"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -233,7 +254,6 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
@@ -244,27 +264,31 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -286,7 +310,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -344,7 +368,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -357,13 +381,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -375,86 +398,49 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="20" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
+    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>